<commit_message>
Labour/plant build-up form, similar-item search, spec differences in levelling, archive project
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ShGswK3SJJeEsEzfdZjprk
</commit_message>
<xml_diff>
--- a/templates/assembly_library_template.xlsx
+++ b/templates/assembly_library_template.xlsx
@@ -9327,7 +9327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U153"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9551,21 +9551,6 @@
           <t>excl</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>bag</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>KSA-ALL</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9658,21 +9643,6 @@
           <t>incl</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>KSA-CENTRAL</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>A.01</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9760,21 +9730,6 @@
           <t>exempt</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>ha</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>KSA-EASTERN</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>A.02</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9827,21 +9782,6 @@
           <t>Unverified</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>KSA-NORTHERN</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>A.03</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9874,21 +9814,6 @@
           <t>subcontract</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>KSA-SOUTHERN</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>A.04</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9916,21 +9841,6 @@
           <t>assembly</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>KSA-WESTERN</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>A.05</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9953,16 +9863,6 @@
           <t>other</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>km</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>A.06</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9978,1124 +9878,6 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>unpriced</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>kva</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>A.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>kw</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>A.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>A.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>length_piece</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>A.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>ls</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>B.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>B.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>B.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>B.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>B.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>nr</t>
-        </is>
-      </c>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>B.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>pair</t>
-        </is>
-      </c>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>B.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>percent</t>
-        </is>
-      </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>B.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>point</t>
-        </is>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>B.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>roll</t>
-        </is>
-      </c>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>B.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>B.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>sheet</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>B.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>B.13</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>tr</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>B.14</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>trip</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>B.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>week</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>B.16</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>B.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>C.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>C.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>C.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>C.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="U36" t="inlineStr">
-        <is>
-          <t>C.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>C.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>C.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>C.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>C.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="U41" t="inlineStr">
-        <is>
-          <t>C.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="U42" t="inlineStr">
-        <is>
-          <t>C.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="U43" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>D.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="U45" t="inlineStr">
-        <is>
-          <t>D.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="U46" t="inlineStr">
-        <is>
-          <t>D.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>D.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>D.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>D.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>D.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>D.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="U52" t="inlineStr">
-        <is>
-          <t>D.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="U53" t="inlineStr">
-        <is>
-          <t>D.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="U54" t="inlineStr">
-        <is>
-          <t>D.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="U55" t="inlineStr">
-        <is>
-          <t>D.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>D.13</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="U57" t="inlineStr">
-        <is>
-          <t>D.14</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="U58" t="inlineStr">
-        <is>
-          <t>D.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="U59" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="U60" t="inlineStr">
-        <is>
-          <t>E.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="U61" t="inlineStr">
-        <is>
-          <t>E.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="U62" t="inlineStr">
-        <is>
-          <t>E.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="U63" t="inlineStr">
-        <is>
-          <t>E.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="U64" t="inlineStr">
-        <is>
-          <t>E.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="U65" t="inlineStr">
-        <is>
-          <t>E.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="U66" t="inlineStr">
-        <is>
-          <t>E.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="U67" t="inlineStr">
-        <is>
-          <t>E.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="U68" t="inlineStr">
-        <is>
-          <t>E.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="U69" t="inlineStr">
-        <is>
-          <t>E.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="U70" t="inlineStr">
-        <is>
-          <t>E.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="U71" t="inlineStr">
-        <is>
-          <t>E.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>E.13</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="U73" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="U74" t="inlineStr">
-        <is>
-          <t>F.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="U75" t="inlineStr">
-        <is>
-          <t>F.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="U76" t="inlineStr">
-        <is>
-          <t>F.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="U77" t="inlineStr">
-        <is>
-          <t>F.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="U78" t="inlineStr">
-        <is>
-          <t>F.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="U79" t="inlineStr">
-        <is>
-          <t>F.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="U80" t="inlineStr">
-        <is>
-          <t>F.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="U81" t="inlineStr">
-        <is>
-          <t>F.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="U82" t="inlineStr">
-        <is>
-          <t>F.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="U83" t="inlineStr">
-        <is>
-          <t>F.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="U84" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="U85" t="inlineStr">
-        <is>
-          <t>G.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="U86" t="inlineStr">
-        <is>
-          <t>G.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="U87" t="inlineStr">
-        <is>
-          <t>G.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="U88" t="inlineStr">
-        <is>
-          <t>G.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="U89" t="inlineStr">
-        <is>
-          <t>G.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="U90" t="inlineStr">
-        <is>
-          <t>G.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="U91" t="inlineStr">
-        <is>
-          <t>G.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="U92" t="inlineStr">
-        <is>
-          <t>G.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="U93" t="inlineStr">
-        <is>
-          <t>G.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="U94" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="U95" t="inlineStr">
-        <is>
-          <t>H.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="U96" t="inlineStr">
-        <is>
-          <t>H.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="U97" t="inlineStr">
-        <is>
-          <t>H.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="U98" t="inlineStr">
-        <is>
-          <t>H.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="U99" t="inlineStr">
-        <is>
-          <t>H.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="U100" t="inlineStr">
-        <is>
-          <t>H.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="U101" t="inlineStr">
-        <is>
-          <t>H.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="U102" t="inlineStr">
-        <is>
-          <t>H.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="U103" t="inlineStr">
-        <is>
-          <t>H.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="U104" t="inlineStr">
-        <is>
-          <t>H.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="U105" t="inlineStr">
-        <is>
-          <t>H.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="U106" t="inlineStr">
-        <is>
-          <t>H.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="U107" t="inlineStr">
-        <is>
-          <t>H.13</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="U108" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="U109" t="inlineStr">
-        <is>
-          <t>I.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="U110" t="inlineStr">
-        <is>
-          <t>I.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="U111" t="inlineStr">
-        <is>
-          <t>I.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="U112" t="inlineStr">
-        <is>
-          <t>I.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="U113" t="inlineStr">
-        <is>
-          <t>I.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="U114" t="inlineStr">
-        <is>
-          <t>I.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="U115" t="inlineStr">
-        <is>
-          <t>I.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="U116" t="inlineStr">
-        <is>
-          <t>I.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="U117" t="inlineStr">
-        <is>
-          <t>I.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="U118" t="inlineStr">
-        <is>
-          <t>I.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="U119" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="U120" t="inlineStr">
-        <is>
-          <t>J.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="U121" t="inlineStr">
-        <is>
-          <t>J.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="U122" t="inlineStr">
-        <is>
-          <t>J.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="U123" t="inlineStr">
-        <is>
-          <t>J.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="U124" t="inlineStr">
-        <is>
-          <t>J.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="U125" t="inlineStr">
-        <is>
-          <t>J.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>J.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="U127" t="inlineStr">
-        <is>
-          <t>J.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="U128" t="inlineStr">
-        <is>
-          <t>J.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="U129" t="inlineStr">
-        <is>
-          <t>J.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="U130" t="inlineStr">
-        <is>
-          <t>J.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="U131" t="inlineStr">
-        <is>
-          <t>J.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="U132" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="U133" t="inlineStr">
-        <is>
-          <t>K.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="U134" t="inlineStr">
-        <is>
-          <t>K.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="U135" t="inlineStr">
-        <is>
-          <t>K.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="U136" t="inlineStr">
-        <is>
-          <t>K.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="U137" t="inlineStr">
-        <is>
-          <t>K.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="U138" t="inlineStr">
-        <is>
-          <t>K.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="U139" t="inlineStr">
-        <is>
-          <t>K.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="U140" t="inlineStr">
-        <is>
-          <t>K.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="U141" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="U142" t="inlineStr">
-        <is>
-          <t>L.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="U143" t="inlineStr">
-        <is>
-          <t>L.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="U144" t="inlineStr">
-        <is>
-          <t>L.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="U145" t="inlineStr">
-        <is>
-          <t>L.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="U146" t="inlineStr">
-        <is>
-          <t>L.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="U147" t="inlineStr">
-        <is>
-          <t>L.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="U148" t="inlineStr">
-        <is>
-          <t>L.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="U149" t="inlineStr">
-        <is>
-          <t>L.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="U150" t="inlineStr">
-        <is>
-          <t>L.09</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="U151" t="inlineStr">
-        <is>
-          <t>L.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="U152" t="inlineStr">
-        <is>
-          <t>L.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="U153" t="inlineStr">
-        <is>
-          <t>L.12</t>
         </is>
       </c>
     </row>

</xml_diff>